<commit_message>
Enhanced UI and improved forensic analysis workflow
</commit_message>
<xml_diff>
--- a/reports/evidence_report.xlsx
+++ b/reports/evidence_report.xlsx
@@ -78,17 +78,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0000B050"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
   </fills>
@@ -659,21 +659,21 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>billing_invoices_2026.csv</t>
+          <t>ehr_case_summary_P001.txt</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>healthcare_data\billing\billing_invoices_2026.csv</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\EHR\ehr_case_summary_P001.txt</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.02</v>
+        <v>1.82</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -697,17 +697,17 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>01915f851ddb7436e4916f196234f243c0f011433fa9539646bca3a148ac1aa5</t>
+          <t>fc6e6ceaee54d233eb0a122cb1ceee2fa7009fa48b9b12088737036f7bd41eee</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>86cad2a532e557907184ad199949ddee</t>
+          <t>30dbc5c86afde117badb70bf2cfbc1bf</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -717,26 +717,26 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Billing &amp; Financial</t>
+          <t>Electronic Health Record</t>
         </is>
       </c>
       <c r="S2" s="2" t="n">
-        <v>4.6898</v>
+        <v>5.0459</v>
       </c>
       <c r="T2" s="2" t="b">
         <v>0</v>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -758,12 +758,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>ehr_case_summary_P001.txt</t>
+          <t>pharmacy_drug_inventory.txt</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>healthcare_data\EHR\ehr_case_summary_P001.txt</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\Pharmacy\pharmacy_drug_inventory.txt</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1.82</v>
+        <v>2.42</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -786,56 +786,56 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-07 12:13:54</t>
+          <t>2026-04-10 11:19:34</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-07 12:13:54</t>
+          <t>2026-04-10 11:19:34</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>fc6e6ceaee54d233eb0a122cb1ceee2fa7009fa48b9b12088737036f7bd41eee</t>
+          <t>7f82a1811f7869bfbec59be7b223ce268b5fb7f7514eade8aec65d378df5a299</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>30dbc5c86afde117badb70bf2cfbc1bf</t>
+          <t>d8eed2b1b83470a8ddb56f53f0ffe461</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Modified After Breach</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>Electronic Health Record</t>
+          <t>Pharmacy &amp; Prescription</t>
         </is>
       </c>
       <c r="S3" s="4" t="n">
-        <v>5.0459</v>
+        <v>4.7317</v>
       </c>
       <c r="T3" s="4" t="b">
         <v>0</v>
       </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -857,21 +857,21 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>billing_payment_summary.txt</t>
+          <t>billing_invoices_2026.csv</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>healthcare_data\billing\billing_payment_summary.txt</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\billing\billing_invoices_2026.csv</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1.8</v>
+        <v>2.02</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -885,41 +885,41 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13 11:23:30</t>
+          <t>2026-04-07 12:13:54</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13 11:23:30</t>
+          <t>2026-04-07 12:13:54</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>25dd2ddb7f4435a684f563ad12eb56ea7730d9d289572388b800b8fd52ccde1f</t>
+          <t>01915f851ddb7436e4916f196234f243c0f011433fa9539646bca3a148ac1aa5</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>1f922ad1dadf8930eca130c5a0c43cd6</t>
+          <t>86cad2a532e557907184ad199949ddee</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Modified After Breach</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
@@ -927,14 +927,14 @@
         </is>
       </c>
       <c r="S4" s="2" t="n">
-        <v>4.6736</v>
+        <v>4.6898</v>
       </c>
       <c r="T4" s="2" t="b">
         <v>0</v>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -956,21 +956,21 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>lab_test_results_2026.csv</t>
+          <t>lab_report_P003_cardiac.txt</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>healthcare_data\lab reports\lab_test_results_2026.csv</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\lab reports\lab_report_P003_cardiac.txt</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2.91</v>
+        <v>2.1</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -994,17 +994,17 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>ef9f2d5b367cbf71c1ddaf1ebd7af7973271ed0fda77eb0a56b149df755f0aaa</t>
+          <t>2733f840c7d6c052b02395ced2cb1584b6b6e85ba310f4cbaba91cf7ab0e6797</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>cd35e3d18d28c56919fabdb451d23a0a</t>
+          <t>1aee86a0efb085a75b9b3030744ffa0b</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -1014,11 +1014,11 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
@@ -1026,14 +1026,14 @@
         </is>
       </c>
       <c r="S5" s="4" t="n">
-        <v>5.1902</v>
+        <v>4.8812</v>
       </c>
       <c r="T5" s="4" t="b">
         <v>0</v>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>pharmacy_drug_inventory.txt</t>
+          <t>billing_payment_summary.txt</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>healthcare_data\Pharmacy\pharmacy_drug_inventory.txt</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\billing\billing_payment_summary.txt</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2.42</v>
+        <v>1.85</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -1083,27 +1083,27 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10 11:19:34</t>
+          <t>2026-04-13 11:23:30</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10 11:19:34</t>
+          <t>2026-04-21 21:33:33</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:31</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>7f82a1811f7869bfbec59be7b223ce268b5fb7f7514eade8aec65d378df5a299</t>
+          <t>aec65b18afc29f37dcd02744d580518a9184d8d127b5f1b32d3fbb70288d6b01</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>d8eed2b1b83470a8ddb56f53f0ffe461</t>
+          <t>2d221627d5d54e344b95a3cca15f1c9c</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
           <t>Modified After Breach</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1121,18 +1121,18 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy &amp; Prescription</t>
+          <t>Billing &amp; Financial</t>
         </is>
       </c>
       <c r="S6" s="2" t="n">
-        <v>4.7317</v>
+        <v>4.7272</v>
       </c>
       <c r="T6" s="2" t="b">
         <v>0</v>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>healthcare_data\EHR\ehr_patient_records.csv</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\EHR\ehr_patient_records.csv</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -1210,7 +1210,7 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1253,12 +1253,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>pharmacy_prescriptions_2026.csv</t>
+          <t>lab_test_results_2026.csv</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>healthcare_data\Pharmacy\pharmacy_prescriptions_2026.csv</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\lab reports\lab_test_results_2026.csv</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3.23</v>
+        <v>2.91</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -1281,56 +1281,56 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10 11:19:34</t>
+          <t>2026-04-07 12:13:54</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10 11:19:34</t>
+          <t>2026-04-07 12:13:54</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>6f91fe9b1a1ccfd7cadc6db1750cbec2829c65d347b98a97b1d5f65e6593c1dd</t>
+          <t>ef9f2d5b367cbf71c1ddaf1ebd7af7973271ed0fda77eb0a56b149df755f0aaa</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>8715ba0958638216b7051221455fafe5</t>
+          <t>cd35e3d18d28c56919fabdb451d23a0a</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Modified After Breach</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy &amp; Prescription</t>
+          <t>Laboratory Report</t>
         </is>
       </c>
       <c r="S8" s="2" t="n">
-        <v>5.1344</v>
+        <v>5.1902</v>
       </c>
       <c r="T8" s="2" t="b">
         <v>0</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1352,21 +1352,21 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>lab_report_P003_cardiac.txt</t>
+          <t>surgery_records_2026.csv</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>healthcare_data\lab reports\lab_report_P003_cardiac.txt</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\Surgery\surgery_records_2026.csv</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>2.1</v>
+        <v>1.54</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -1380,56 +1380,56 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-04-07 12:13:54</t>
+          <t>2026-04-10 11:19:34</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>2026-04-07 12:13:54</t>
+          <t>2026-04-10 11:19:34</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2733f840c7d6c052b02395ced2cb1584b6b6e85ba310f4cbaba91cf7ab0e6797</t>
+          <t>ddd36e955cdd522a7d075bb64c958a736dbfe21d5fcba8adf40739def94fca89</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>1aee86a0efb085a75b9b3030744ffa0b</t>
+          <t>adca6c3fa1a4046c35860b575efda123</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Modified After Breach</t>
         </is>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Laboratory Report</t>
+          <t>Structured Healthcare Dataset</t>
         </is>
       </c>
       <c r="S9" s="4" t="n">
-        <v>4.8812</v>
+        <v>5.1705</v>
       </c>
       <c r="T9" s="4" t="b">
         <v>0</v>
       </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>surgery_records_2026.csv</t>
+          <t>pharmacy_prescriptions_2026.csv</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>healthcare_data\Surgery\surgery_records_2026.csv</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\Pharmacy\pharmacy_prescriptions_2026.csv</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1.54</v>
+        <v>3.23</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -1489,17 +1489,17 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>ddd36e955cdd522a7d075bb64c958a736dbfe21d5fcba8adf40739def94fca89</t>
+          <t>6f91fe9b1a1ccfd7cadc6db1750cbec2829c65d347b98a97b1d5f65e6593c1dd</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>adca6c3fa1a4046c35860b575efda123</t>
+          <t>8715ba0958638216b7051221455fafe5</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1507,7 +1507,7 @@
           <t>Modified After Breach</t>
         </is>
       </c>
-      <c r="P10" s="6" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1517,18 +1517,18 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Structured Healthcare Dataset</t>
+          <t>Pharmacy &amp; Prescription</t>
         </is>
       </c>
       <c r="S10" s="2" t="n">
-        <v>5.1705</v>
+        <v>5.1344</v>
       </c>
       <c r="T10" s="2" t="b">
         <v>0</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>healthcare_data\Surgery\surgery_report_P003_angioplasty.txt</t>
+          <t>C:\Users\nirma\OneDrive\Desktop\cli and web final\healthcare_data\Surgery\surgery_report_P003_angioplasty.txt</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:08</t>
+          <t>2026-04-28 19:37:22</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -1606,7 +1606,7 @@
           <t>Modified After Breach</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21 20:54:24</t>
+          <t>2026-04-28 19:37:48</t>
         </is>
       </c>
     </row>

</xml_diff>